<commit_message>
Re-run ZE1 list with corrected row 17 and document analysis recipe.
Use Schmitt + TTRI (expected 3) for all pairs, write ANALYSIS_METHOD.md,
and refresh summary/JSON after the fixed 右腓腸肌 a10 Delsys reference.

Co-authored-by: frankrita0728-coder <frankrita0728-coder@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/pairing_results/2609-21_ZE1_list/source_list.xlsx
+++ b/data/pairing_results/2609-21_ZE1_list/source_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zenta\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F3AB67-45CC-4661-97E7-F0628C132146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3606295D-414A-43AD-822A-9A0894609DAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="90">
   <si>
     <t>分析部位</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -380,6 +380,10 @@
   </si>
   <si>
     <t>2609-09 frank 左腓腸肌_a09_褲XL_疲勞3.csv</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2609-09 frank右腓腸肌(Delsys)_with_a10_2.csv</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1005,7 +1009,7 @@
         <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
         <v>39</v>

</xml_diff>